<commit_message>
daily auto push: 2026-08-28 23:00 UTC
</commit_message>
<xml_diff>
--- a/excel/sei1.xlsx
+++ b/excel/sei1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2429"/>
+  <dimension ref="A1:D2430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43401,19 +43401,19 @@
     <row r="2388">
       <c r="A2388" t="inlineStr">
         <is>
-          <t>2026/12/29</t>
+          <t>2026/08/29</t>
         </is>
       </c>
       <c r="B2388" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C2388" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D2388" t="n">
-        <v>88</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2389">
@@ -43428,10 +43428,10 @@
         </is>
       </c>
       <c r="C2389" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D2389" t="n">
-        <v>99</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2390">
@@ -43446,10 +43446,10 @@
         </is>
       </c>
       <c r="C2390" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D2390" t="n">
-        <v>81</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2391">
@@ -43464,28 +43464,28 @@
         </is>
       </c>
       <c r="C2391" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D2391" t="n">
-        <v>85</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2392">
       <c r="A2392" t="inlineStr">
         <is>
-          <t>2026/12/30</t>
+          <t>2026/12/29</t>
         </is>
       </c>
       <c r="B2392" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C2392" t="n">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D2392" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2393">
@@ -43500,10 +43500,10 @@
         </is>
       </c>
       <c r="C2393" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D2393" t="n">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2394">
@@ -43518,10 +43518,10 @@
         </is>
       </c>
       <c r="C2394" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D2394" t="n">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2395">
@@ -43536,10 +43536,10 @@
         </is>
       </c>
       <c r="C2395" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D2395" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2396">
@@ -43554,10 +43554,10 @@
         </is>
       </c>
       <c r="C2396" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D2396" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2397">
@@ -43572,28 +43572,28 @@
         </is>
       </c>
       <c r="C2397" t="n">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D2397" t="n">
-        <v>108</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2398">
       <c r="A2398" t="inlineStr">
         <is>
-          <t>2026/12/31</t>
+          <t>2026/12/30</t>
         </is>
       </c>
       <c r="B2398" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C2398" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D2398" t="n">
-        <v>114</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2399">
@@ -43608,10 +43608,10 @@
         </is>
       </c>
       <c r="C2399" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D2399" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2400">
@@ -43626,7 +43626,7 @@
         </is>
       </c>
       <c r="C2400" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D2400" t="n">
         <v>120</v>
@@ -43644,10 +43644,10 @@
         </is>
       </c>
       <c r="C2401" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D2401" t="n">
-        <v>201</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2402">
@@ -43662,10 +43662,10 @@
         </is>
       </c>
       <c r="C2402" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D2402" t="n">
-        <v>130</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2403">
@@ -43680,28 +43680,28 @@
         </is>
       </c>
       <c r="C2403" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D2403" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2404">
       <c r="A2404" t="inlineStr">
         <is>
-          <t>2027/01/01</t>
+          <t>2026/12/31</t>
         </is>
       </c>
       <c r="B2404" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C2404" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D2404" t="n">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2405">
@@ -43716,10 +43716,10 @@
         </is>
       </c>
       <c r="C2405" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D2405" t="n">
-        <v>119</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2406">
@@ -43734,10 +43734,10 @@
         </is>
       </c>
       <c r="C2406" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D2406" t="n">
-        <v>133</v>
+        <v>119</v>
       </c>
     </row>
     <row r="2407">
@@ -43752,10 +43752,10 @@
         </is>
       </c>
       <c r="C2407" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D2407" t="n">
-        <v>109</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2408">
@@ -43770,28 +43770,28 @@
         </is>
       </c>
       <c r="C2408" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D2408" t="n">
-        <v>120</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2409">
       <c r="A2409" t="inlineStr">
         <is>
-          <t>2027/01/02</t>
+          <t>2027/01/01</t>
         </is>
       </c>
       <c r="B2409" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C2409" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="D2409" t="n">
-        <v>105</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2410">
@@ -43806,10 +43806,10 @@
         </is>
       </c>
       <c r="C2410" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D2410" t="n">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2411">
@@ -43824,10 +43824,10 @@
         </is>
       </c>
       <c r="C2411" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D2411" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2412">
@@ -43842,10 +43842,10 @@
         </is>
       </c>
       <c r="C2412" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D2412" t="n">
-        <v>132</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2413">
@@ -43860,10 +43860,10 @@
         </is>
       </c>
       <c r="C2413" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D2413" t="n">
-        <v>145</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2414">
@@ -43878,10 +43878,10 @@
         </is>
       </c>
       <c r="C2414" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D2414" t="n">
-        <v>157</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2415">
@@ -43896,28 +43896,28 @@
         </is>
       </c>
       <c r="C2415" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D2415" t="n">
-        <v>165</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2416">
       <c r="A2416" t="inlineStr">
         <is>
-          <t>2027/01/03</t>
+          <t>2027/01/02</t>
         </is>
       </c>
       <c r="B2416" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C2416" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D2416" t="n">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2417">
@@ -43932,10 +43932,10 @@
         </is>
       </c>
       <c r="C2417" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D2417" t="n">
-        <v>192</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2418">
@@ -43950,10 +43950,10 @@
         </is>
       </c>
       <c r="C2418" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D2418" t="n">
-        <v>189</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2419">
@@ -43968,10 +43968,10 @@
         </is>
       </c>
       <c r="C2419" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D2419" t="n">
-        <v>201</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2420">
@@ -43986,7 +43986,7 @@
         </is>
       </c>
       <c r="C2420" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D2420" t="n">
         <v>201</v>
@@ -44004,7 +44004,7 @@
         </is>
       </c>
       <c r="C2421" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D2421" t="n">
         <v>201</v>
@@ -44022,28 +44022,28 @@
         </is>
       </c>
       <c r="C2422" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D2422" t="n">
-        <v>194</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2423">
       <c r="A2423" t="inlineStr">
         <is>
-          <t>2027/01/04</t>
+          <t>2027/01/03</t>
         </is>
       </c>
       <c r="B2423" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C2423" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D2423" t="n">
-        <v>164</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2424">
@@ -44058,10 +44058,10 @@
         </is>
       </c>
       <c r="C2424" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D2424" t="n">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2425">
@@ -44076,10 +44076,10 @@
         </is>
       </c>
       <c r="C2425" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D2425" t="n">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2426">
@@ -44094,10 +44094,10 @@
         </is>
       </c>
       <c r="C2426" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D2426" t="n">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2427">
@@ -44112,28 +44112,28 @@
         </is>
       </c>
       <c r="C2427" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D2427" t="n">
-        <v>127</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2428">
       <c r="A2428" t="inlineStr">
         <is>
-          <t>2027/01/05</t>
+          <t>2027/01/04</t>
         </is>
       </c>
       <c r="B2428" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C2428" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="D2428" t="n">
-        <v>118</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2429">
@@ -44148,9 +44148,27 @@
         </is>
       </c>
       <c r="C2429" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2429" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2430">
+      <c r="A2430" t="inlineStr">
+        <is>
+          <t>2027/01/05</t>
+        </is>
+      </c>
+      <c r="B2430" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C2430" t="n">
         <v>7</v>
       </c>
-      <c r="D2429" t="n">
+      <c r="D2430" t="n">
         <v>127</v>
       </c>
     </row>

</xml_diff>